<commit_message>
CORE-000031 edit: update to include RS
</commit_message>
<xml_diff>
--- a/rules/CORE-000031/negative/01/data/unit-test-coreid-CG0659-negative 1.xlsx
+++ b/rules/CORE-000031/negative/01/data/unit-test-coreid-CG0659-negative 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000031\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8393279F-362A-482C-9EDA-CCE2F5B8578F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DCC5A49-3556-4E8C-8CB4-5D7263636585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,27 @@
     <sheet name="Validation" sheetId="3" r:id="rId3"/>
     <sheet name="ft.xpt" sheetId="4" r:id="rId4"/>
     <sheet name="rs.xpt" sheetId="5" r:id="rId5"/>
+    <sheet name="vs.xpt" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="143">
   <si>
     <t>Product</t>
   </si>
@@ -342,13 +356,124 @@
   </si>
   <si>
     <t>Disease Response and Clinical Classification</t>
+  </si>
+  <si>
+    <t>vs.xpt</t>
+  </si>
+  <si>
+    <t>Vital Signs</t>
+  </si>
+  <si>
+    <t>VSSEQ</t>
+  </si>
+  <si>
+    <t>VSTESTCD</t>
+  </si>
+  <si>
+    <t>VSTEST</t>
+  </si>
+  <si>
+    <t>VSPOS</t>
+  </si>
+  <si>
+    <t>VSORRES</t>
+  </si>
+  <si>
+    <t>VSORRESU</t>
+  </si>
+  <si>
+    <t>VSSTRESC</t>
+  </si>
+  <si>
+    <t>VSSTRESN</t>
+  </si>
+  <si>
+    <t>VSSTRESU</t>
+  </si>
+  <si>
+    <t>VSSTAT</t>
+  </si>
+  <si>
+    <t>VSLOC</t>
+  </si>
+  <si>
+    <t>VSLOBXFL</t>
+  </si>
+  <si>
+    <t>VSREPNUM</t>
+  </si>
+  <si>
+    <t>VSDTC</t>
+  </si>
+  <si>
+    <t>VSDY</t>
+  </si>
+  <si>
+    <t>Vital Signs Test Short Name</t>
+  </si>
+  <si>
+    <t>Vital Signs Test Name</t>
+  </si>
+  <si>
+    <t>Vital Signs Position of Subject</t>
+  </si>
+  <si>
+    <t>Original Units</t>
+  </si>
+  <si>
+    <t>Standard Units</t>
+  </si>
+  <si>
+    <t>Completion Status</t>
+  </si>
+  <si>
+    <t>Location of Vital Signs Measurement</t>
+  </si>
+  <si>
+    <t>Date/Time of Measurements</t>
+  </si>
+  <si>
+    <t>Study Day of Vital Signs</t>
+  </si>
+  <si>
+    <t>VS</t>
+  </si>
+  <si>
+    <t>DIABP</t>
+  </si>
+  <si>
+    <t>Diastolic Blood Pressure</t>
+  </si>
+  <si>
+    <t>STANDING</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>mmHg</t>
+  </si>
+  <si>
+    <t>SCREENING 1</t>
+  </si>
+  <si>
+    <t>2012-11-23</t>
+  </si>
+  <si>
+    <t>VSEVAL</t>
+  </si>
+  <si>
+    <t>sdtmct</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -375,6 +500,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -435,9 +565,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -456,6 +585,11 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,14 +892,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
     </row>
@@ -775,6 +909,14 @@
       </c>
       <c r="B2" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -784,14 +926,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>5</v>
       </c>
     </row>
@@ -809,6 +951,14 @@
       </c>
       <c r="B3" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -821,26 +971,29 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>13</v>
       </c>
     </row>
@@ -895,349 +1048,349 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="T2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="U2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="V2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="W2" s="3" t="s">
+      <c r="W2" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="L3" s="3" t="s">
+      <c r="E3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="N3" s="3" t="s">
+      <c r="M3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="O3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="P3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="S3" s="3" t="s">
+      <c r="P3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="S3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="T3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="U3" s="3" t="s">
+      <c r="T3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="U3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="V3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="W3" s="3" t="s">
+      <c r="V3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="W3" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>12</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-      <c r="C4" s="3">
-        <v>8</v>
-      </c>
-      <c r="D4" s="3">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3">
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2">
         <v>7</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <v>23</v>
       </c>
-      <c r="G4" s="3">
-        <v>8</v>
-      </c>
-      <c r="H4" s="3">
+      <c r="G4" s="2">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2">
         <v>200</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="2">
         <v>200</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="2">
         <v>12</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="2">
         <v>200</v>
       </c>
-      <c r="L4" s="3">
-        <v>8</v>
-      </c>
-      <c r="M4" s="3">
+      <c r="L4" s="2">
+        <v>8</v>
+      </c>
+      <c r="M4" s="2">
         <v>1</v>
       </c>
-      <c r="N4" s="3">
-        <v>8</v>
-      </c>
-      <c r="O4" s="3">
-        <v>8</v>
-      </c>
-      <c r="P4" s="3">
+      <c r="N4" s="2">
+        <v>8</v>
+      </c>
+      <c r="O4" s="2">
+        <v>8</v>
+      </c>
+      <c r="P4" s="2">
         <v>200</v>
       </c>
-      <c r="Q4" s="3">
+      <c r="Q4" s="2">
         <v>9</v>
       </c>
-      <c r="R4" s="3">
+      <c r="R4" s="2">
         <v>19</v>
       </c>
-      <c r="S4" s="3">
-        <v>8</v>
-      </c>
-      <c r="T4" s="3">
+      <c r="S4" s="2">
+        <v>8</v>
+      </c>
+      <c r="T4" s="2">
         <v>200</v>
       </c>
-      <c r="U4" s="3">
-        <v>8</v>
-      </c>
-      <c r="V4" s="3">
+      <c r="U4" s="2">
+        <v>8</v>
+      </c>
+      <c r="V4" s="2">
         <v>200</v>
       </c>
-      <c r="W4" s="3">
+      <c r="W4" s="2">
         <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4" t="s">
+      <c r="L5" s="3"/>
+      <c r="M5" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="4">
+      <c r="N5" s="3">
         <v>1</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="3">
         <v>2</v>
       </c>
-      <c r="P5" s="4" t="s">
+      <c r="P5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="Q5" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="R5" s="4" t="s">
+      <c r="R5" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="S5" s="4">
+      <c r="S5" s="3">
         <v>-2</v>
       </c>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1250,280 +1403,615 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="R1" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="R1" s="7" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="2" spans="1:18" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="R2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2">
+        <v>37</v>
+      </c>
+      <c r="G4" s="2">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2">
+        <v>198</v>
+      </c>
+      <c r="I4" s="2">
+        <v>8</v>
+      </c>
+      <c r="J4" s="2">
+        <v>8</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2">
+        <v>8</v>
+      </c>
+      <c r="M4" s="2">
+        <v>200</v>
+      </c>
+      <c r="N4" s="2">
+        <v>9</v>
+      </c>
+      <c r="O4" s="2">
+        <v>10</v>
+      </c>
+      <c r="P4" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>200</v>
+      </c>
+      <c r="R4" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="105" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="J5" s="3">
+        <v>1</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L5" s="3">
+        <v>3</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="P5" s="3">
+        <v>1</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB7A739F-9C1B-4DDD-93ED-B1F033E664F9}">
+  <dimension ref="A1:V5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="V2" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="3" t="s">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J3" s="3" t="s">
+      <c r="E3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="P3" s="3" t="s">
+      <c r="Q3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="Q3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="R3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>12</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-      <c r="C4" s="3">
-        <v>8</v>
-      </c>
-      <c r="D4" s="3">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3">
-        <v>8</v>
-      </c>
-      <c r="F4" s="3">
-        <v>37</v>
-      </c>
-      <c r="G4" s="3">
-        <v>7</v>
-      </c>
-      <c r="H4" s="3">
-        <v>198</v>
-      </c>
-      <c r="I4" s="3">
-        <v>8</v>
-      </c>
-      <c r="J4" s="3">
-        <v>8</v>
-      </c>
-      <c r="K4" s="3">
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2">
+        <v>24</v>
+      </c>
+      <c r="G4" s="2">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2">
+        <v>8</v>
+      </c>
+      <c r="I4" s="2">
+        <v>9</v>
+      </c>
+      <c r="J4" s="2">
+        <v>200</v>
+      </c>
+      <c r="K4" s="2">
+        <v>8</v>
+      </c>
+      <c r="L4" s="2">
+        <v>9</v>
+      </c>
+      <c r="M4" s="2">
+        <v>8</v>
+      </c>
+      <c r="N4" s="2">
+        <v>11</v>
+      </c>
+      <c r="O4" s="2">
         <v>1</v>
       </c>
-      <c r="L4" s="3">
-        <v>8</v>
-      </c>
-      <c r="M4" s="3">
+      <c r="P4" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>8</v>
+      </c>
+      <c r="R4" s="2">
         <v>200</v>
       </c>
-      <c r="N4" s="3">
+      <c r="S4" s="2">
         <v>9</v>
       </c>
-      <c r="O4" s="3">
+      <c r="T4" s="2">
         <v>10</v>
       </c>
-      <c r="P4" s="3">
-        <v>8</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>19</v>
-      </c>
-      <c r="R4" s="3">
+      <c r="U4" s="2">
+        <v>8</v>
+      </c>
+      <c r="V4" s="2">
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="105" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:22" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="J5" s="4">
+      <c r="E5" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K5" s="3">
+        <v>71</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q5" s="3">
         <v>1</v>
       </c>
-      <c r="K5" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="L5" s="4">
-        <v>3</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="N5" s="4" t="s">
+      <c r="R5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="S5" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="O5" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="P5" s="4">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>102</v>
+      <c r="T5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="U5" s="3">
+        <v>-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CORE-000031 edit: rule verified and made fully executable with updated rule logic and test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000031/negative/01/data/unit-test-coreid-CG0659-negative 1.xlsx
+++ b/rules/CORE-000031/negative/01/data/unit-test-coreid-CG0659-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000031\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DCC5A49-3556-4E8C-8CB4-5D7263636585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D4B1EF-19F4-492A-990A-1A0741F6A037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -466,7 +466,7 @@
     <t>sdtmct</t>
   </si>
   <si>
-    <t>2026-03-27</t>
+    <t>2025-03-28</t>
   </si>
 </sst>
 </file>

</xml_diff>